<commit_message>
Expand Russian thematic hashtags for all 50 Ozon SKUs and document checks
</commit_message>
<xml_diff>
--- a/ozon/phase1/20261029-2310/Ozon_phase1_核对工作簿_50SKU.xlsx
+++ b/ozon/phase1/20261029-2310/Ozon_phase1_核对工作簿_50SKU.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每款与合卡" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待确认事项" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐SKU源值与换算" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主题标签核对" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'说明与检查'!$A$1:$B$13</definedName>
@@ -21,6 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'每款与合卡'!$A$1:$F$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'待确认事项'!$A$1:$E$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'逐SKU源值与换算'!$A$1:$F$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'主题标签核对'!$A$1:$E$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -9238,4 +9240,1303 @@
   <autoFilter ref="A1:F51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>原SKU</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>新SKU</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>标签数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>完整主题标签</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>依据及限制</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2018YF044</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH044</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2018YF043</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH043</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2018YF042</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH042</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2018YF041QH</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH041QH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2018YF041PT</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH041PT</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2018YF041</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH041</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2018YF040</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH040</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2018YF039</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH039</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2018YF038</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH038</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2018YF037</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH037</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2018YF036</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH036</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2018YF035-1</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH035-1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2018YF035-2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH035-2</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2018YF035-3</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH035-3</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2018YF034</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH034</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #автопутешествия #активный_отдых #комфорт_в_пути #поездки_на_природу</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2018YF033</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH033</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #автопутешествия #активный_отдых #комфорт_в_пути #поездки_на_природу</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2018YF032RL</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH032RL</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2018YF032</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH032</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2018YF031</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH031</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2018YF029</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH029</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2018YF028</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH028</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2018YF027</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH027</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2018YF026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH026</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2018YF025</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH025</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2018YF024PT</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH024PT</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2018YF023</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH023</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2018YF021</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH021</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2018YF019</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH019</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #жизнь_за_рулём #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2018YF018</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH018</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #жизнь_за_рулём #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2018YF017</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH017</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2018YF016</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH016</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2018YF015</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH015</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2018YF014</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH014</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2018YF013</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH013</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2018YF012</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH012</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2018YF011</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH011</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2018YF010</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH010</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2018YF009</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH009</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2018YF008</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH008</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2018YF007-010</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH007-010</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2018YF007</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH007</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2018YF006</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH006</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2018YF005</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH005</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2018YF004</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH004</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2018YF003-006</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH003-006</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2018YF003</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH003</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #самостоятельный_ремонт #гаражный_ремонт #восстановление #повседневные_поездки</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2018YF002Y</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH002Y</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2018YF002S</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH002S</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2018YF002B</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH002B</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #стиль_в_деталях #автоэстетика #обновление_образа #индивидуальный_стиль</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2018YF001</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH001</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>#автолюбитель #автожизнь #гараж #автопроект #гаражные_будни #своими_руками #уход_за_автомобилем #вторая_жизнь #автопутешествия #активный_отдых #комфорт_в_пути #поездки_на_природу</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>俄文主题/用途标签；未验证实时热度，不承诺爆款或流量；未加入品牌、商品名称或规格</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E51"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>